<commit_message>
Practicing IF functions of SUM and COUNT
</commit_message>
<xml_diff>
--- a/1.4. EXCEL  SECTION - Basic Formulas and Functions/1.4.2.1 Excel - Basic Mathematical Functions working file Working.xlsx
+++ b/1.4. EXCEL  SECTION - Basic Formulas and Functions/1.4.2.1 Excel - Basic Mathematical Functions working file Working.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rittiv/Documents/GitHub/Projects-Data/1.4. EXCEL  SECTION - Basic Formulas and Functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473B6C67-B5CB-BC4F-8ABA-3C9C79E27DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAB3312-5363-A643-9276-484F872878DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15140" yWindow="680" windowWidth="15120" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -93,9 +93,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -188,7 +189,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -199,16 +200,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -223,8 +215,14 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="5" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="5" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="7" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -526,28 +524,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="5" t="s">
         <v>14</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5">
+      <c r="I1" s="4">
         <f>COUNT(F2:F30)</f>
         <v>29</v>
       </c>
@@ -555,22 +553,22 @@
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="10">
+      <c r="A2" s="7">
         <v>2222686</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="7">
         <v>36</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="11">
+      <c r="C2" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="8">
         <v>2.5</v>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="7">
         <v>480</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="11">
         <f>D2*E2</f>
         <v>1200</v>
       </c>
@@ -580,29 +578,29 @@
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="10">
+      <c r="A3" s="7">
         <v>9137942</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="7">
         <v>50</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="11">
+      <c r="C3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="8">
         <v>1.5</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="7">
         <v>610</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="11">
         <f t="shared" ref="F3:F30" si="0">D3*E3</f>
         <v>915</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="4">
         <f>SUM(E2:E30)</f>
         <v>14870</v>
       </c>
@@ -610,29 +608,29 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="10">
+      <c r="A4" s="7">
         <v>2591591</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="7">
         <v>70</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="11">
-        <v>3</v>
-      </c>
-      <c r="E4" s="10">
+      <c r="D4" s="8">
+        <v>3</v>
+      </c>
+      <c r="E4" s="7">
         <v>490</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="11">
         <f t="shared" si="0"/>
         <v>1470</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="9">
         <f>SUM(F2:F30)</f>
         <v>32515</v>
       </c>
@@ -640,22 +638,22 @@
       <c r="K4" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="10">
+      <c r="A5" s="7">
         <v>5727287</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="7">
         <v>23</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="11">
-        <v>3</v>
-      </c>
-      <c r="E5" s="10">
+      <c r="D5" s="8">
+        <v>3</v>
+      </c>
+      <c r="E5" s="7">
         <v>530</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="11">
         <f t="shared" si="0"/>
         <v>1590</v>
       </c>
@@ -665,22 +663,22 @@
       <c r="K5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="10">
+      <c r="A6" s="7">
         <v>6696095</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="7">
         <v>80</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="11">
+      <c r="C6" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="8">
         <v>1.5</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="7">
         <v>520</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="11">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
@@ -696,130 +694,166 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="10">
+      <c r="A7" s="7">
         <v>2071811</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="7">
         <v>39</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="11">
-        <v>3</v>
-      </c>
-      <c r="E7" s="10">
+      <c r="D7" s="8">
+        <v>3</v>
+      </c>
+      <c r="E7" s="7">
         <v>400</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="11">
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="6"/>
+      <c r="I7" s="4">
+        <f>COUNTIF($C$2:$C$30, H7)</f>
+        <v>13</v>
+      </c>
+      <c r="J7" s="4">
+        <f>SUMIF($C$2:$C$30, H7, $E$2:$E$30)</f>
+        <v>7330</v>
+      </c>
+      <c r="K7" s="10">
+        <f>SUMIF($C$2:$C$30, H7, $F$2:$F$30)</f>
+        <v>10995</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="10">
+      <c r="A8" s="7">
         <v>1681422</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="7">
         <v>18</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="11">
+      <c r="C8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="8">
         <v>2.5</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="7">
         <v>240</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="11">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="6"/>
+      <c r="I8" s="4">
+        <f t="shared" ref="I8:I10" si="1">COUNTIF($C$2:$C$30, H8)</f>
+        <v>6</v>
+      </c>
+      <c r="J8" s="4">
+        <f t="shared" ref="J8:J9" si="2">SUMIF($C$2:$C$30, H8, $E$2:$E$30)</f>
+        <v>2200</v>
+      </c>
+      <c r="K8" s="10">
+        <f t="shared" ref="K8:K9" si="3">SUMIF($C$2:$C$30, H8, $F$2:$F$30)</f>
+        <v>5500</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="10">
+      <c r="A9" s="7">
         <v>7923665</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="7">
         <v>28</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="11">
-        <v>3</v>
-      </c>
-      <c r="E9" s="10">
+      <c r="D9" s="8">
+        <v>3</v>
+      </c>
+      <c r="E9" s="7">
         <v>770</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="11">
         <f t="shared" si="0"/>
         <v>2310</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="6"/>
+      <c r="I9" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="J9" s="4">
+        <f t="shared" si="2"/>
+        <v>5340</v>
+      </c>
+      <c r="K9" s="10">
+        <f t="shared" si="3"/>
+        <v>16020</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="10">
+      <c r="A10" s="7">
         <v>6495990</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="7">
         <v>66</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="11">
+      <c r="C10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="8">
         <v>2.5</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="7">
         <v>120</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="11">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="4"/>
+      <c r="I10" s="4">
+        <f>SUM(I7:I9)</f>
+        <v>29</v>
+      </c>
+      <c r="J10" s="4">
+        <f>SUM(J7:J9)</f>
+        <v>14870</v>
+      </c>
+      <c r="K10" s="9">
+        <f>SUM(K7:K9)</f>
+        <v>32515</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="10">
+      <c r="A11" s="7">
         <v>2884971</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="7">
         <v>76</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="11">
+      <c r="C11" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="8">
         <v>1.5</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="7">
         <v>260</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="11">
         <f t="shared" si="0"/>
         <v>390</v>
       </c>
@@ -829,406 +863,406 @@
       <c r="K11" s="1"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="10">
+      <c r="A12" s="7">
         <v>3104248</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="7">
         <v>76</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="11">
+      <c r="C12" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="8">
         <v>1.5</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="7">
         <v>380</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="11">
         <f t="shared" si="0"/>
         <v>570</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I12" s="5"/>
+      <c r="I12" s="4"/>
       <c r="J12" s="2"/>
       <c r="K12" s="1"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="10">
+      <c r="A13" s="7">
         <v>6591759</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="7">
         <v>45</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="11">
-        <v>3</v>
-      </c>
-      <c r="E13" s="10">
+      <c r="D13" s="8">
+        <v>3</v>
+      </c>
+      <c r="E13" s="7">
         <v>220</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="11">
         <f t="shared" si="0"/>
         <v>660</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="10">
+      <c r="A14" s="7">
         <v>1654144</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="7">
         <v>29</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" s="11">
+      <c r="C14" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="8">
         <v>1.5</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="7">
         <v>120</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="11">
         <f t="shared" si="0"/>
         <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="10">
+      <c r="A15" s="7">
         <v>5838000</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="7">
         <v>98</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" s="11">
+      <c r="C15" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" s="8">
         <v>2.5</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="7">
         <v>580</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="11">
         <f t="shared" si="0"/>
         <v>1450</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="10">
+      <c r="A16" s="7">
         <v>2613499</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="7">
         <v>46</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="11">
-        <v>3</v>
-      </c>
-      <c r="E16" s="10">
+      <c r="D16" s="8">
+        <v>3</v>
+      </c>
+      <c r="E16" s="7">
         <v>830</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="11">
         <f t="shared" si="0"/>
         <v>2490</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="10">
+      <c r="A17" s="7">
         <v>6452597</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="7">
         <v>14</v>
       </c>
-      <c r="C17" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D17" s="11">
+      <c r="C17" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="8">
         <v>1.5</v>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="7">
         <v>940</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="11">
         <f t="shared" si="0"/>
         <v>1410</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="10">
+      <c r="A18" s="7">
         <v>3597671</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="7">
         <v>72</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D18" s="11">
+      <c r="C18" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="8">
         <v>1.5</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="7">
         <v>860</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="11">
         <f t="shared" si="0"/>
         <v>1290</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="10">
+      <c r="A19" s="7">
         <v>3497037</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="7">
         <v>23</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D19" s="11">
+      <c r="C19" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="8">
         <v>1.5</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="7">
         <v>990</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="11">
         <f t="shared" si="0"/>
         <v>1485</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="10">
+      <c r="A20" s="7">
         <v>7245825</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="7">
         <v>60</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D20" s="11">
+      <c r="C20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="8">
         <v>2.5</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="7">
         <v>420</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="11">
         <f t="shared" si="0"/>
         <v>1050</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="10">
+      <c r="A21" s="7">
         <v>3752341</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="7">
         <v>98</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="11">
-        <v>3</v>
-      </c>
-      <c r="E21" s="10">
+      <c r="D21" s="8">
+        <v>3</v>
+      </c>
+      <c r="E21" s="7">
         <v>680</v>
       </c>
-      <c r="F21" s="12">
+      <c r="F21" s="11">
         <f t="shared" si="0"/>
         <v>2040</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="10">
+      <c r="A22" s="7">
         <v>2228642</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="7">
         <v>28</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D22" s="11">
+      <c r="C22" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="8">
         <v>1.5</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E22" s="7">
         <v>500</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="11">
         <f t="shared" si="0"/>
         <v>750</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="10">
+      <c r="A23" s="7">
         <v>6308184</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="7">
         <v>97</v>
       </c>
-      <c r="C23" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="11">
+      <c r="C23" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="8">
         <v>1.5</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="7">
         <v>420</v>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="11">
         <f t="shared" si="0"/>
         <v>630</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="10">
+      <c r="A24" s="7">
         <v>7322687</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="7">
         <v>56</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="11">
+      <c r="C24" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="8">
         <v>1.5</v>
       </c>
-      <c r="E24" s="10">
+      <c r="E24" s="7">
         <v>570</v>
       </c>
-      <c r="F24" s="12">
+      <c r="F24" s="11">
         <f t="shared" si="0"/>
         <v>855</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="10">
+      <c r="A25" s="7">
         <v>6253313</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="7">
         <v>19</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="11">
-        <v>3</v>
-      </c>
-      <c r="E25" s="10">
+      <c r="D25" s="8">
+        <v>3</v>
+      </c>
+      <c r="E25" s="7">
         <v>250</v>
       </c>
-      <c r="F25" s="12">
+      <c r="F25" s="11">
         <f t="shared" si="0"/>
         <v>750</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="10">
+      <c r="A26" s="7">
         <v>7136401</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="7">
         <v>16</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D26" s="11">
+      <c r="C26" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="8">
         <v>1.5</v>
       </c>
-      <c r="E26" s="10">
+      <c r="E26" s="7">
         <v>920</v>
       </c>
-      <c r="F26" s="12">
+      <c r="F26" s="11">
         <f t="shared" si="0"/>
         <v>1380</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="10">
+      <c r="A27" s="7">
         <v>5693278</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="7">
         <v>17</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D27" s="11">
+      <c r="C27" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" s="8">
         <v>2.5</v>
       </c>
-      <c r="E27" s="10">
+      <c r="E27" s="7">
         <v>360</v>
       </c>
-      <c r="F27" s="12">
+      <c r="F27" s="11">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="10">
+      <c r="A28" s="7">
         <v>2637109</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="7">
         <v>98</v>
       </c>
-      <c r="C28" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D28" s="11">
+      <c r="C28" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D28" s="8">
         <v>1.5</v>
       </c>
-      <c r="E28" s="10">
+      <c r="E28" s="7">
         <v>240</v>
       </c>
-      <c r="F28" s="12">
+      <c r="F28" s="11">
         <f t="shared" si="0"/>
         <v>360</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="10">
+      <c r="A29" s="7">
         <v>4298027</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="7">
         <v>96</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="11">
-        <v>3</v>
-      </c>
-      <c r="E29" s="10">
+      <c r="D29" s="8">
+        <v>3</v>
+      </c>
+      <c r="E29" s="7">
         <v>450</v>
       </c>
-      <c r="F29" s="12">
+      <c r="F29" s="11">
         <f t="shared" si="0"/>
         <v>1350</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="10">
+      <c r="A30" s="7">
         <v>1698653</v>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="7">
         <v>64</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="11">
-        <v>3</v>
-      </c>
-      <c r="E30" s="10">
+      <c r="D30" s="8">
+        <v>3</v>
+      </c>
+      <c r="E30" s="7">
         <v>720</v>
       </c>
-      <c r="F30" s="12">
+      <c r="F30" s="11">
         <f t="shared" si="0"/>
         <v>2160</v>
       </c>

</xml_diff>